<commit_message>
feat(recipes): xuất/nhập Excel hỗ trợ Tùy chọn thêm + ghi đè giá khi trùng tên
- Thêm sheet "Tùy chọn thêm" và "Công thức tùy chọn" vào import/export (trước
  đây import không có cách nào tạo product_extras hàng loạt).
- Thêm nút xuất toàn bộ thiết lập hiện tại của địa chỉ ra đúng layout file
  import, để sửa trực tiếp trong Excel rồi nạp lại thay vì gõ tay.
- Sản phẩm/Nguyên liệu/Topping/Tùy chọn thêm trùng tên khi import giờ CẬP
  NHẬT giá (Nguyên liệu cập nhật cả đơn vị) thay vì bị bỏ qua như trước.
- Chuẩn hoá NFC khi so khớp tên (Excel/macOS có thể lưu dấu ở dạng tổ hợp
  khác với dữ liệu gõ qua trình duyệt) — tránh tạo trùng vì 2 tên nhìn giống
  hệt nhau nhưng khác encoding.
- Khi commit lỗi giữa chừng, đồng bộ lại state + buộc chọn lại file trước khi
  thử lại, để tránh tạo trùng dữ liệu đã ghi được ở lần thử trước.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/mau-nhap-lieu.xlsx
+++ b/public/templates/mau-nhap-lieu.xlsx
@@ -10,6 +10,8 @@
     <sheet name="Topping" sheetId="5" r:id="rId5"/>
     <sheet name="Công thức Topping" sheetId="6" r:id="rId6"/>
     <sheet name="Topping áp dụng món" sheetId="7" r:id="rId7"/>
+    <sheet name="Tùy chọn thêm" sheetId="8" r:id="rId8"/>
+    <sheet name="Công thức tùy chọn" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -403,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -417,12 +419,12 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2. 1 sản phẩm/nguyên liệu/topping chỉ nên xuất hiện 1 lần ở sheet định nghĩa của nó (Sản phẩm/Nguyên liệu/Topping) — trùng tên sẽ bị báo lỗi.</v>
+        <v>2. Sản phẩm/Nguyên liệu/Topping: trùng tên với dữ liệu đã có sẽ CẬP NHẬT giá (Nguyên liệu cập nhật cả đơn vị) — không tạo trùng.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>3. Sheet Công thức, Công thức Topping, Topping áp dụng món: lặp lại tên món/topping ở nhiều dòng nếu có nhiều nguyên liệu/liên kết.</v>
+        <v>3. Sheet Công thức, Công thức Topping, Công thức tùy chọn, Topping áp dụng món: lặp lại tên món/topping/tùy chọn ở nhiều dòng nếu có nhiều nguyên liệu/liên kết.</v>
       </c>
     </row>
     <row r="5">
@@ -432,12 +434,22 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>5. Giá bán/Giá vốn là số nguyên (VNĐ), không kèm chữ "đ" hay dấu phẩy.</v>
+        <v>5. Giá bán/Giá vốn/Giá là số nguyên (VNĐ), không kèm chữ "đ" hay dấu phẩy.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>6. Sheet Tùy chọn thêm: mỗi dòng là 1 tùy chọn (size, topping rời...) gắn vào 1 món, có giá riêng. Cột Tự động chọn: "có" nếu muốn tùy chọn này tự bật sẵn khi khách chọn món, để trống nếu không.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>7. Sheet Topping áp dụng món: ghi đè TOÀN BỘ danh sách món của mỗi topping trong file — món cũ không có trong file sẽ bị gỡ liên kết.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -736,4 +748,88 @@
     <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Tên món</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Tên tùy chọn</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Giá</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Tự động chọn</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Cà Phê Sữa</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Size L</v>
+      </c>
+      <c r="C2">
+        <v>5000</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Tên món</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Tên tùy chọn</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Tên nguyên liệu</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Số lượng</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Đơn vị</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Cà Phê Sữa</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Size L</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Cà phê</v>
+      </c>
+      <c r="D2">
+        <v>10</v>
+      </c>
+      <c r="E2" t="str">
+        <v>g</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>